<commit_message>
Reshape arena to circle (radius-based), arrange shop balls in a ring, fold joker slots into grid hex coords, add camera zoom slider
- Arena: replace arena_width/height with arena_radius; floor becomes a disc mesh and walls become a ring of cuboid segments; wave spawn and jumper sample inside the circle.
- Shop: rune balls sit on a ring (SHOP_BALL_RING_RADIUS) and shop floors become two discs.
- Runes: drop RuneSource::Joker and JokerSlots resource; jokers are now designated hex coords on the grid (JOKER_COORDS, is_joker_slot); grid radius shrunk from 3 to 2.
- Dev menu: add CameraZoom resource + slider (separate from camera angle), extracted shared slider_drag_t helper; Win Wave button only in combat dev menu.
</commit_message>
<xml_diff>
--- a/assets/balance.xlsx
+++ b/assets/balance.xlsx
@@ -1180,7 +1180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="24.04" customWidth="1" style="11" min="1" max="1"/>
@@ -1223,138 +1223,124 @@
     <row r="3" ht="15" customHeight="1" s="7">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>arena_width</t>
+          <t>arena_radius</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>1800</v>
+        <v>900</v>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>fixed arena width</t>
+          <t>fixed arena radius</t>
         </is>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="7">
       <c r="A4" s="11" t="inlineStr">
         <is>
-          <t>arena_height</t>
+          <t>coins_per_kill</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>1800</v>
+        <v>1</v>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>fixed arena height</t>
+          <t>coin drops per mob kill</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="7">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>coins_per_kill</t>
+          <t>coin_attraction_duration</t>
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>coin drops per mob kill</t>
+          <t>coin flight duration toward player (s)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="7">
       <c r="A6" s="11" t="inlineStr">
         <is>
-          <t>coin_attraction_duration</t>
+          <t>rune_joker_probability</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>coin flight duration toward player (s)</t>
+          <t>chance shop slot rolls as joker</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="7">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>rune_joker_probability</t>
+          <t>rune_tier_weight_common</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>0.1</v>
+        <v>60</v>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>chance shop slot rolls as joker</t>
+          <t>common-tier weight in shop roll</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="7">
       <c r="A8" s="11" t="inlineStr">
         <is>
-          <t>rune_tier_weight_common</t>
+          <t>rune_tier_weight_rare</t>
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>common-tier weight in shop roll</t>
+          <t>rare-tier weight in shop roll</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="7">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>rune_tier_weight_rare</t>
+          <t>rune_reroll_base_cost</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>rare-tier weight in shop roll</t>
+          <t>cost of first reroll per shop session</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="7">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>rune_reroll_base_cost</t>
+          <t>rune_reroll_cost_step</t>
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>cost of first reroll per shop session</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="7">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>rune_reroll_cost_step</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
           <t>per-reroll cost increase</t>
         </is>
       </c>
     </row>
+    <row r="11" ht="15" customHeight="1" s="7"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Switch waves to timed continuous spawning, grow arena per wave
- Replace WaveDef.max_concurrent (u32) with spawn_interval (f32); spawn
  one enemy per accumulated interval until the wave timer ends, no cap.
- Order apply_wave_config after reset_wave_state so the StartWaveEvent
  pair is deterministic (was racy on wasm; first wave never spawned).
- Extend Waves sheet to 40 rows; hp/damage multipliers grow geometrically
  to 3x by wave 40; spawn_interval ramps 2.5s to 0.3s.
- Halve base damage column in Mobs sheet.
- Shrink default arena (Globals.arena_radius 900 to 450), zoom camera in
  1.5x (CameraZoom default height 1080 to 720).
- Grow arena radius +50 per wave, capped at 1000; floor was already
  reactive, walls now respawn when CurrentArenaSize changes.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/balance.xlsx
+++ b/assets/balance.xlsx
@@ -453,7 +453,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D2" s="6" t="n">
         <v>120</v>
@@ -479,7 +479,7 @@
         <v>25</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D3" s="6" t="inlineStr"/>
       <c r="E3" s="6" t="n">
@@ -505,7 +505,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="D4" s="6" t="n">
         <v>300</v>
@@ -531,7 +531,7 @@
         <v>10</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>400</v>
@@ -561,7 +561,7 @@
         <v>15</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>1200</v>
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11.12" customWidth="1" style="9" min="2" max="2"/>
@@ -604,506 +604,916 @@
     <col width="18.85" customWidth="1" style="6" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="7">
-      <c r="A1" s="13" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>wave</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>unlocks</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>enemy_variety</t>
         </is>
       </c>
-      <c r="D1" s="13" t="inlineStr">
-        <is>
-          <t>max_concurrent</t>
-        </is>
-      </c>
-      <c r="E1" s="13" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>spawn_interval</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
         <is>
           <t>hp_multiplier</t>
         </is>
       </c>
-      <c r="F1" s="13" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>damage_multiplier</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="7">
-      <c r="A2" s="6" t="n">
+    <row r="2">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>slime_small</t>
         </is>
       </c>
-      <c r="C2" s="6" t="n">
+      <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="7">
-      <c r="A3" s="6" t="n">
+      <c r="D2">
+        <v>2.5</v>
+      </c>
+      <c r="E2">
+        <v>1.0</v>
+      </c>
+      <c r="F2">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>ghost</t>
         </is>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="C3">
         <v>2</v>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D3">
+        <v>2.3</v>
+      </c>
+      <c r="E3">
+        <v>1.0286</v>
+      </c>
+      <c r="F3">
+        <v>1.0286</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>2.12</v>
+      </c>
+      <c r="E4">
+        <v>1.058</v>
+      </c>
+      <c r="F4">
+        <v>1.058</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>jumper</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>1.95</v>
+      </c>
+      <c r="E5">
+        <v>1.0882</v>
+      </c>
+      <c r="F5">
+        <v>1.0882</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>1.79</v>
+      </c>
+      <c r="E6">
+        <v>1.1193</v>
+      </c>
+      <c r="F6">
+        <v>1.1193</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="E3" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="7">
-      <c r="A4" s="6" t="n">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C7">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="inlineStr"/>
-      <c r="C4" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="6" t="n">
+      <c r="D7">
+        <v>1.65</v>
+      </c>
+      <c r="E7">
+        <v>1.1512</v>
+      </c>
+      <c r="F7">
+        <v>1.1512</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>tower</t>
+        </is>
+      </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>1.52</v>
+      </c>
+      <c r="E8">
+        <v>1.1841</v>
+      </c>
+      <c r="F8">
+        <v>1.1841</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9">
+        <v>1.39</v>
+      </c>
+      <c r="E9">
+        <v>1.218</v>
+      </c>
+      <c r="F9">
+        <v>1.218</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>1.28</v>
+      </c>
+      <c r="E10">
+        <v>1.2528</v>
+      </c>
+      <c r="F10">
+        <v>1.2528</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C11">
         <v>4</v>
       </c>
-      <c r="F4" s="6" t="n">
-        <v>1.44</v>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="7">
-      <c r="A5" s="6" t="n">
+      <c r="D11">
+        <v>1.18</v>
+      </c>
+      <c r="E11">
+        <v>1.2886</v>
+      </c>
+      <c r="F11">
+        <v>1.2886</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C12">
         <v>4</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>jumper</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>1.728</v>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="7">
-      <c r="A6" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr"/>
-      <c r="C6" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="E6" s="6" t="n">
+      <c r="D12">
+        <v>1.09</v>
+      </c>
+      <c r="E12">
+        <v>1.3254</v>
+      </c>
+      <c r="F12">
+        <v>1.3254</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+      <c r="D13">
+        <v>1.0</v>
+      </c>
+      <c r="E13">
+        <v>1.3632</v>
+      </c>
+      <c r="F13">
+        <v>1.3632</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>spinner</t>
+        </is>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+      <c r="D14">
+        <v>0.92</v>
+      </c>
+      <c r="E14">
+        <v>1.4022</v>
+      </c>
+      <c r="F14">
+        <v>1.4022</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C15">
+        <v>5</v>
+      </c>
+      <c r="D15">
+        <v>0.85</v>
+      </c>
+      <c r="E15">
+        <v>1.4422</v>
+      </c>
+      <c r="F15">
+        <v>1.4422</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C16">
+        <v>5</v>
+      </c>
+      <c r="D16">
+        <v>0.78</v>
+      </c>
+      <c r="E16">
+        <v>1.4835</v>
+      </c>
+      <c r="F16">
+        <v>1.4835</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
         <v>16</v>
       </c>
-      <c r="F6" s="6" t="n">
-        <v>2.0736</v>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="7">
-      <c r="A7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="6" t="inlineStr"/>
-      <c r="C7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="E7" s="6" t="n">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C17">
+        <v>5</v>
+      </c>
+      <c r="D17">
+        <v>0.72</v>
+      </c>
+      <c r="E17">
+        <v>1.5258</v>
+      </c>
+      <c r="F17">
+        <v>1.5258</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C18">
+        <v>5</v>
+      </c>
+      <c r="D18">
+        <v>0.66</v>
+      </c>
+      <c r="E18">
+        <v>1.5694</v>
+      </c>
+      <c r="F18">
+        <v>1.5694</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C19">
+        <v>5</v>
+      </c>
+      <c r="D19">
+        <v>0.61</v>
+      </c>
+      <c r="E19">
+        <v>1.6143</v>
+      </c>
+      <c r="F19">
+        <v>1.6143</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C20">
+        <v>5</v>
+      </c>
+      <c r="D20">
+        <v>0.56</v>
+      </c>
+      <c r="E20">
+        <v>1.6604</v>
+      </c>
+      <c r="F20">
+        <v>1.6604</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C21">
+        <v>5</v>
+      </c>
+      <c r="D21">
+        <v>0.51</v>
+      </c>
+      <c r="E21">
+        <v>1.7078</v>
+      </c>
+      <c r="F21">
+        <v>1.7078</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C22">
+        <v>5</v>
+      </c>
+      <c r="D22">
+        <v>0.47</v>
+      </c>
+      <c r="E22">
+        <v>1.7566</v>
+      </c>
+      <c r="F22">
+        <v>1.7566</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C23">
+        <v>5</v>
+      </c>
+      <c r="D23">
+        <v>0.43</v>
+      </c>
+      <c r="E23">
+        <v>1.8068</v>
+      </c>
+      <c r="F23">
+        <v>1.8068</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C24">
+        <v>5</v>
+      </c>
+      <c r="D24">
+        <v>0.4</v>
+      </c>
+      <c r="E24">
+        <v>1.8584</v>
+      </c>
+      <c r="F24">
+        <v>1.8584</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C25">
+        <v>5</v>
+      </c>
+      <c r="D25">
+        <v>0.37</v>
+      </c>
+      <c r="E25">
+        <v>1.9115</v>
+      </c>
+      <c r="F25">
+        <v>1.9115</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C26">
+        <v>5</v>
+      </c>
+      <c r="D26">
+        <v>0.34</v>
+      </c>
+      <c r="E26">
+        <v>1.9661</v>
+      </c>
+      <c r="F26">
+        <v>1.9661</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C27">
+        <v>5</v>
+      </c>
+      <c r="D27">
+        <v>0.31</v>
+      </c>
+      <c r="E27">
+        <v>2.0223</v>
+      </c>
+      <c r="F27">
+        <v>2.0223</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C28">
+        <v>5</v>
+      </c>
+      <c r="D28">
+        <v>0.3</v>
+      </c>
+      <c r="E28">
+        <v>2.0801</v>
+      </c>
+      <c r="F28">
+        <v>2.0801</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C29">
+        <v>5</v>
+      </c>
+      <c r="D29">
+        <v>0.3</v>
+      </c>
+      <c r="E29">
+        <v>2.1395</v>
+      </c>
+      <c r="F29">
+        <v>2.1395</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C30">
+        <v>5</v>
+      </c>
+      <c r="D30">
+        <v>0.3</v>
+      </c>
+      <c r="E30">
+        <v>2.2006</v>
+      </c>
+      <c r="F30">
+        <v>2.2006</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C31">
+        <v>5</v>
+      </c>
+      <c r="D31">
+        <v>0.3</v>
+      </c>
+      <c r="E31">
+        <v>2.2635</v>
+      </c>
+      <c r="F31">
+        <v>2.2635</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C32">
+        <v>5</v>
+      </c>
+      <c r="D32">
+        <v>0.3</v>
+      </c>
+      <c r="E32">
+        <v>2.3282</v>
+      </c>
+      <c r="F32">
+        <v>2.3282</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
         <v>32</v>
       </c>
-      <c r="F7" s="6" t="n">
-        <v>2.48832</v>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="7">
-      <c r="A8" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>tower</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>64</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>2.985984</v>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="7">
-      <c r="A9" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="6" t="inlineStr"/>
-      <c r="C9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>128</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>3.5831808</v>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="7">
-      <c r="A10" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="6" t="inlineStr"/>
-      <c r="C10" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>256</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>4.29981696</v>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="7">
-      <c r="A11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr"/>
-      <c r="C11" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>512</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>5.159780352</v>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="7">
-      <c r="A12" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="6" t="inlineStr"/>
-      <c r="C12" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>1024</v>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>6.1917364224</v>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="7">
-      <c r="A13" s="6" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="6" t="inlineStr"/>
-      <c r="C13" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="E13" s="6" t="n">
-        <v>2048</v>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>7.43008370688</v>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="7">
-      <c r="A14" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>spinner</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D14" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="E14" s="6" t="n">
-        <v>4096</v>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>8.916100448256</v>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="7">
-      <c r="A15" s="6" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="6" t="inlineStr"/>
-      <c r="C15" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D15" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="E15" s="6" t="n">
-        <v>8192</v>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>10.6993205379072</v>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="7">
-      <c r="A16" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="6" t="inlineStr"/>
-      <c r="C16" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>16384</v>
-      </c>
-      <c r="F16" s="6" t="n">
-        <v>12.83918464548864</v>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="7">
-      <c r="A17" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="6" t="inlineStr"/>
-      <c r="C17" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="E17" s="6" t="n">
-        <v>32768</v>
-      </c>
-      <c r="F17" s="6" t="n">
-        <v>15.40702157458637</v>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="7">
-      <c r="A18" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="6" t="inlineStr"/>
-      <c r="C18" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="E18" s="6" t="n">
-        <v>65536</v>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>18.48842588950364</v>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="7">
-      <c r="A19" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="6" t="inlineStr"/>
-      <c r="C19" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="E19" s="6" t="n">
-        <v>131072</v>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>22.18611106740437</v>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="7">
-      <c r="A20" s="6" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="6" t="inlineStr"/>
-      <c r="C20" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D20" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="E20" s="6" t="n">
-        <v>262144</v>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>26.62333328088524</v>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="7">
-      <c r="A21" s="6" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="6" t="inlineStr"/>
-      <c r="C21" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D21" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="E21" s="6" t="n">
-        <v>524288</v>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>31.9479999370623</v>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="7">
-      <c r="A22" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr"/>
-      <c r="C22" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D22" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="E22" s="6" t="n">
-        <v>1048576</v>
-      </c>
-      <c r="F22" s="6" t="n">
-        <v>38.33759992447475</v>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="7">
-      <c r="A23" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="6" t="inlineStr"/>
-      <c r="C23" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D23" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="E23" s="6" t="n">
-        <v>2097152</v>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>46.0051199093697</v>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="7">
-      <c r="A24" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="6" t="inlineStr"/>
-      <c r="C24" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D24" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="E24" s="6" t="n">
-        <v>4194304</v>
-      </c>
-      <c r="F24" s="6" t="n">
-        <v>55.20614389124364</v>
-      </c>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="7">
-      <c r="A25" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="6" t="inlineStr"/>
-      <c r="C25" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D25" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="E25" s="6" t="n">
-        <v>8388608</v>
-      </c>
-      <c r="F25" s="6" t="n">
-        <v>66.24737266949238</v>
-      </c>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="7">
-      <c r="A26" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="6" t="inlineStr"/>
-      <c r="C26" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D26" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="E26" s="6" t="n">
-        <v>16777216</v>
-      </c>
-      <c r="F26" s="6" t="n">
-        <v>79.49684720339086</v>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C33">
+        <v>5</v>
+      </c>
+      <c r="D33">
+        <v>0.3</v>
+      </c>
+      <c r="E33">
+        <v>2.3947</v>
+      </c>
+      <c r="F33">
+        <v>2.3947</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C34">
+        <v>5</v>
+      </c>
+      <c r="D34">
+        <v>0.3</v>
+      </c>
+      <c r="E34">
+        <v>2.4631</v>
+      </c>
+      <c r="F34">
+        <v>2.4631</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C35">
+        <v>5</v>
+      </c>
+      <c r="D35">
+        <v>0.3</v>
+      </c>
+      <c r="E35">
+        <v>2.5335</v>
+      </c>
+      <c r="F35">
+        <v>2.5335</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C36">
+        <v>5</v>
+      </c>
+      <c r="D36">
+        <v>0.3</v>
+      </c>
+      <c r="E36">
+        <v>2.6059</v>
+      </c>
+      <c r="F36">
+        <v>2.6059</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C37">
+        <v>5</v>
+      </c>
+      <c r="D37">
+        <v>0.3</v>
+      </c>
+      <c r="E37">
+        <v>2.6803</v>
+      </c>
+      <c r="F37">
+        <v>2.6803</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C38">
+        <v>5</v>
+      </c>
+      <c r="D38">
+        <v>0.3</v>
+      </c>
+      <c r="E38">
+        <v>2.7569</v>
+      </c>
+      <c r="F38">
+        <v>2.7569</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C39">
+        <v>5</v>
+      </c>
+      <c r="D39">
+        <v>0.3</v>
+      </c>
+      <c r="E39">
+        <v>2.8357</v>
+      </c>
+      <c r="F39">
+        <v>2.8357</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C40">
+        <v>5</v>
+      </c>
+      <c r="D40">
+        <v>0.3</v>
+      </c>
+      <c r="E40">
+        <v>2.9167</v>
+      </c>
+      <c r="F40">
+        <v>2.9167</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C41">
+        <v>5</v>
+      </c>
+      <c r="D41">
+        <v>0.3</v>
+      </c>
+      <c r="E41">
+        <v>3.0</v>
+      </c>
+      <c r="F41">
+        <v>3.0</v>
       </c>
     </row>
   </sheetData>
@@ -1227,7 +1637,7 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>900</v>
+        <v>450</v>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>

</xml_diff>